<commit_message>
add top_k as parameter
</commit_message>
<xml_diff>
--- a/results/evaluation/answers/eval_rag_combined.xlsx
+++ b/results/evaluation/answers/eval_rag_combined.xlsx
@@ -435,17 +435,17 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>a_hu</t>
+          <t>a_hu_top5</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>a_qwen2.5</t>
+          <t>a_qwen2.5_top5</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>a_llama3.1</t>
+          <t>a_llama3.1_top5</t>
         </is>
       </c>
     </row>
@@ -3452,7 +3452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3463,10 +3463,15 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>top_k</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>EM</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>F1</t>
         </is>
@@ -3479,9 +3484,12 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C2" t="n">
         <v>0.62</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>0.6836666666666666</v>
       </c>
     </row>
@@ -3492,9 +3500,12 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" t="n">
         <v>0.54</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>0.6033333333333334</v>
       </c>
     </row>
@@ -3505,9 +3516,12 @@
         </is>
       </c>
       <c r="B4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" t="n">
         <v>0.52</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>0.5875714285714285</v>
       </c>
     </row>

</xml_diff>